<commit_message>
update gameplay mock up
</commit_message>
<xml_diff>
--- a/XmlData/Datas/cheeseDictionary.xlsx
+++ b/XmlData/Datas/cheeseDictionary.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\yinya\Documents\unityProjects\GGJ2026\XmlData\Datas\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3FA97E79-B006-416A-A217-1D8124CF095E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6B3205BB-238A-4D76-ABAB-A8989FD240F7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="4635" yWindow="2595" windowWidth="21600" windowHeight="11175" xr2:uid="{53B3FBB6-B116-408D-BCC0-737AAAC6C9D0}"/>
+    <workbookView xWindow="-23940" yWindow="-360" windowWidth="21600" windowHeight="11180" xr2:uid="{53B3FBB6-B116-408D-BCC0-737AAAC6C9D0}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="27" uniqueCount="20">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="30" uniqueCount="21">
   <si>
     <t>##var</t>
     <phoneticPr fontId="1" type="noConversion"/>
@@ -91,6 +91,9 @@
   </si>
   <si>
     <t>list,WordContent</t>
+  </si>
+  <si>
+    <t>CheeseWord_test_03</t>
   </si>
 </sst>
 </file>
@@ -196,16 +199,16 @@
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="3" xfId="0" applyFill="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="3" xfId="0" applyFill="1" applyBorder="1">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -522,7 +525,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8D4CF470-E9E0-44FF-BA6C-71B5C42FB7B2}">
-  <dimension ref="A1:I6"/>
+  <dimension ref="A1:I7"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="7" bestFit="1" customWidth="1"/>
@@ -546,50 +549,50 @@
       <c r="C1" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="D1" s="4" t="s">
+      <c r="D1" s="6" t="s">
         <v>18</v>
       </c>
-      <c r="E1" s="4"/>
-      <c r="F1" s="4"/>
-      <c r="G1" s="4"/>
-      <c r="H1" s="4"/>
-      <c r="I1" s="4"/>
+      <c r="E1" s="6"/>
+      <c r="F1" s="6"/>
+      <c r="G1" s="6"/>
+      <c r="H1" s="6"/>
+      <c r="I1" s="6"/>
     </row>
-    <row r="2" spans="1:9" s="5" customFormat="1">
-      <c r="A2" s="5" t="s">
+    <row r="2" spans="1:9" s="4" customFormat="1">
+      <c r="A2" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="B2" s="5" t="s">
+      <c r="B2" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="C2" s="5" t="s">
+      <c r="C2" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="D2" s="6" t="s">
+      <c r="D2" s="7" t="s">
         <v>19</v>
       </c>
-      <c r="E2" s="6"/>
-      <c r="F2" s="6"/>
-      <c r="G2" s="6"/>
-      <c r="H2" s="6"/>
-      <c r="I2" s="6"/>
+      <c r="E2" s="7"/>
+      <c r="F2" s="7"/>
+      <c r="G2" s="7"/>
+      <c r="H2" s="7"/>
+      <c r="I2" s="7"/>
     </row>
     <row r="3" spans="1:9" s="1" customFormat="1">
       <c r="A3" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="D3" s="7">
+      <c r="D3" s="5">
         <v>0</v>
       </c>
-      <c r="E3" s="7"/>
-      <c r="F3" s="7">
+      <c r="E3" s="5"/>
+      <c r="F3" s="5">
         <v>1</v>
       </c>
-      <c r="G3" s="7"/>
-      <c r="H3" s="7">
+      <c r="G3" s="5"/>
+      <c r="H3" s="5">
         <v>2</v>
       </c>
-      <c r="I3" s="7"/>
+      <c r="I3" s="5"/>
     </row>
     <row r="4" spans="1:9" s="2" customFormat="1">
       <c r="A4" s="2" t="s">
@@ -654,6 +657,20 @@
         <v>13</v>
       </c>
       <c r="E6" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="7" spans="1:9">
+      <c r="B7">
+        <v>3</v>
+      </c>
+      <c r="C7" t="s">
+        <v>20</v>
+      </c>
+      <c r="D7" t="s">
+        <v>13</v>
+      </c>
+      <c r="E7" t="s">
         <v>8</v>
       </c>
     </row>

</xml_diff>

<commit_message>
spaces fixed for sprites
</commit_message>
<xml_diff>
--- a/XmlData/Datas/cheeseDictionary.xlsx
+++ b/XmlData/Datas/cheeseDictionary.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29530"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24334"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\yinya\Documents\unityProjects\GGJ2026\XmlData\Datas\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Emil\Desktop\projects\GGJ2026\XmlData\Datas\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6B3205BB-238A-4D76-ABAB-A8989FD240F7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CD994E8B-4734-4BAF-A66E-4612823A8A66}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-23940" yWindow="-360" windowWidth="21600" windowHeight="11180" xr2:uid="{53B3FBB6-B116-408D-BCC0-737AAAC6C9D0}"/>
+    <workbookView xWindow="4170" yWindow="5070" windowWidth="28800" windowHeight="15885" xr2:uid="{53B3FBB6-B116-408D-BCC0-737AAAC6C9D0}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -20,12 +20,15 @@
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
     </ext>
+    <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
+      <xlwcv:version setVersion="1"/>
+    </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="30" uniqueCount="21">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="38" uniqueCount="25">
   <si>
     <t>##var</t>
     <phoneticPr fontId="1" type="noConversion"/>
@@ -94,6 +97,18 @@
   </si>
   <si>
     <t>CheeseWord_test_03</t>
+  </si>
+  <si>
+    <t>Asset Notfound</t>
+  </si>
+  <si>
+    <t>Missing Person</t>
+  </si>
+  <si>
+    <t>Asset_Notfound</t>
+  </si>
+  <si>
+    <t>Missing_Person</t>
   </si>
 </sst>
 </file>
@@ -229,9 +244,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
-    <a:clrScheme name="Office 2013 - 2022">
+    <a:clrScheme name="Office">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -269,7 +284,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office 2013 - 2022">
+    <a:fontScheme name="Office">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -375,7 +390,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office 2013 - 2022">
+    <a:fmtScheme name="Office">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -517,7 +532,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -525,12 +540,12 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8D4CF470-E9E0-44FF-BA6C-71B5C42FB7B2}">
-  <dimension ref="A1:I7"/>
+  <dimension ref="A1:I24"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="7" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="3.42578125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="20.140625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="27.28515625" customWidth="1"/>
     <col min="4" max="4" width="12.28515625" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="15.140625" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="12.28515625" bestFit="1" customWidth="1"/>
@@ -672,6 +687,115 @@
       </c>
       <c r="E7" t="s">
         <v>8</v>
+      </c>
+    </row>
+    <row r="8" spans="1:9">
+      <c r="B8">
+        <v>4</v>
+      </c>
+      <c r="C8" t="s">
+        <v>23</v>
+      </c>
+      <c r="D8" t="s">
+        <v>13</v>
+      </c>
+      <c r="E8" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="9" spans="1:9">
+      <c r="B9">
+        <v>5</v>
+      </c>
+      <c r="C9" t="s">
+        <v>24</v>
+      </c>
+      <c r="D9" t="s">
+        <v>13</v>
+      </c>
+      <c r="E9" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="10" spans="1:9">
+      <c r="B10">
+        <v>6</v>
+      </c>
+      <c r="D10" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="11" spans="1:9">
+      <c r="B11">
+        <v>7</v>
+      </c>
+      <c r="D11" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="12" spans="1:9">
+      <c r="B12">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="13" spans="1:9">
+      <c r="B13">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="14" spans="1:9">
+      <c r="B14">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="15" spans="1:9">
+      <c r="B15">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="16" spans="1:9">
+      <c r="B16">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="17" spans="2:2">
+      <c r="B17">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="18" spans="2:2">
+      <c r="B18">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="19" spans="2:2">
+      <c r="B19">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="20" spans="2:2">
+      <c r="B20">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="21" spans="2:2">
+      <c r="B21">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="22" spans="2:2">
+      <c r="B22">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="23" spans="2:2">
+      <c r="B23">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="24" spans="2:2">
+      <c r="B24">
+        <v>20</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
food dictionary images + updates
</commit_message>
<xml_diff>
--- a/XmlData/Datas/cheeseDictionary.xlsx
+++ b/XmlData/Datas/cheeseDictionary.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24334"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\yinya\Documents\unityProjects\GGJ2026\XmlData\Datas\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Emil\Desktop\projects\GGJ2026\XmlData\Datas\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2ADC2451-C038-4DD9-88DA-6D06D697C6D1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{634AF970-E859-4399-A306-6AFB9BEE3043}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-25710" yWindow="-1210" windowWidth="25820" windowHeight="15500" xr2:uid="{53B3FBB6-B116-408D-BCC0-737AAAC6C9D0}"/>
+    <workbookView xWindow="38280" yWindow="5235" windowWidth="29040" windowHeight="16440" xr2:uid="{53B3FBB6-B116-408D-BCC0-737AAAC6C9D0}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -20,12 +20,15 @@
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
     </ext>
+    <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
+      <xlwcv:version setVersion="1"/>
+    </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="125" uniqueCount="63">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="119" uniqueCount="62">
   <si>
     <t>##var</t>
     <phoneticPr fontId="1" type="noConversion"/>
@@ -151,9 +154,6 @@
   </si>
   <si>
     <t>Frozen</t>
-  </si>
-  <si>
-    <t>Chewy</t>
   </si>
   <si>
     <t>Burnt</t>
@@ -355,9 +355,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
-    <a:clrScheme name="Office 2013 - 2022">
+    <a:clrScheme name="Office">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -395,7 +395,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office 2013 - 2022">
+    <a:fontScheme name="Office">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -501,7 +501,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office 2013 - 2022">
+    <a:fmtScheme name="Office">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -643,7 +643,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -651,7 +651,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8D4CF470-E9E0-44FF-BA6C-71B5C42FB7B2}">
-  <dimension ref="A1:I36"/>
+  <dimension ref="A1:I34"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="7" bestFit="1" customWidth="1"/>
@@ -955,13 +955,13 @@
         <v>13</v>
       </c>
       <c r="C17" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="D17" t="s">
         <v>37</v>
       </c>
       <c r="E17" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
     </row>
     <row r="18" spans="2:5">
@@ -983,13 +983,13 @@
         <v>15</v>
       </c>
       <c r="C19" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="D19" t="s">
         <v>37</v>
       </c>
       <c r="E19" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
     </row>
     <row r="20" spans="2:5">
@@ -997,13 +997,13 @@
         <v>16</v>
       </c>
       <c r="C20" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="D20" t="s">
         <v>37</v>
       </c>
       <c r="E20" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
     </row>
     <row r="21" spans="2:5">
@@ -1011,13 +1011,13 @@
         <v>17</v>
       </c>
       <c r="C21" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="D21" t="s">
-        <v>37</v>
+        <v>10</v>
       </c>
       <c r="E21" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
     </row>
     <row r="22" spans="2:5">
@@ -1025,13 +1025,13 @@
         <v>18</v>
       </c>
       <c r="C22" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="D22" t="s">
-        <v>37</v>
+        <v>10</v>
       </c>
       <c r="E22" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
     </row>
     <row r="23" spans="2:5">
@@ -1039,13 +1039,13 @@
         <v>19</v>
       </c>
       <c r="C23" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="D23" t="s">
         <v>10</v>
       </c>
       <c r="E23" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
     </row>
     <row r="24" spans="2:5">
@@ -1053,13 +1053,13 @@
         <v>20</v>
       </c>
       <c r="C24" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="D24" t="s">
         <v>10</v>
       </c>
       <c r="E24" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
     </row>
     <row r="25" spans="2:5">
@@ -1067,13 +1067,13 @@
         <v>21</v>
       </c>
       <c r="C25" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="D25" t="s">
         <v>10</v>
       </c>
       <c r="E25" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
     </row>
     <row r="26" spans="2:5">
@@ -1081,13 +1081,13 @@
         <v>22</v>
       </c>
       <c r="C26" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="D26" t="s">
-        <v>10</v>
+        <v>47</v>
       </c>
       <c r="E26" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
     </row>
     <row r="27" spans="2:5">
@@ -1095,13 +1095,13 @@
         <v>23</v>
       </c>
       <c r="C27" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="D27" t="s">
         <v>10</v>
       </c>
       <c r="E27" t="s">
-        <v>47</v>
+        <v>51</v>
       </c>
     </row>
     <row r="28" spans="2:5">
@@ -1109,13 +1109,13 @@
         <v>24</v>
       </c>
       <c r="C28" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="D28" t="s">
-        <v>48</v>
+        <v>10</v>
       </c>
       <c r="E28" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
     </row>
     <row r="29" spans="2:5">
@@ -1123,10 +1123,10 @@
         <v>25</v>
       </c>
       <c r="C29" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="D29" t="s">
-        <v>10</v>
+        <v>47</v>
       </c>
       <c r="E29" t="s">
         <v>52</v>
@@ -1137,13 +1137,13 @@
         <v>26</v>
       </c>
       <c r="C30" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="D30" t="s">
         <v>10</v>
       </c>
       <c r="E30" t="s">
-        <v>51</v>
+        <v>54</v>
       </c>
     </row>
     <row r="31" spans="2:5">
@@ -1151,13 +1151,13 @@
         <v>27</v>
       </c>
       <c r="C31" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="D31" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="E31" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
     </row>
     <row r="32" spans="2:5">
@@ -1165,13 +1165,13 @@
         <v>28</v>
       </c>
       <c r="C32" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="D32" t="s">
         <v>10</v>
       </c>
       <c r="E32" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
     </row>
     <row r="33" spans="2:5">
@@ -1179,13 +1179,13 @@
         <v>29</v>
       </c>
       <c r="C33" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="D33" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="E33" t="s">
-        <v>56</v>
+        <v>60</v>
       </c>
     </row>
     <row r="34" spans="2:5">
@@ -1193,41 +1193,13 @@
         <v>30</v>
       </c>
       <c r="C34" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="D34" t="s">
         <v>10</v>
       </c>
       <c r="E34" t="s">
         <v>57</v>
-      </c>
-    </row>
-    <row r="35" spans="2:5">
-      <c r="B35">
-        <v>31</v>
-      </c>
-      <c r="C35" t="s">
-        <v>59</v>
-      </c>
-      <c r="D35" t="s">
-        <v>48</v>
-      </c>
-      <c r="E35" t="s">
-        <v>61</v>
-      </c>
-    </row>
-    <row r="36" spans="2:5">
-      <c r="B36">
-        <v>32</v>
-      </c>
-      <c r="C36" t="s">
-        <v>60</v>
-      </c>
-      <c r="D36" t="s">
-        <v>10</v>
-      </c>
-      <c r="E36" t="s">
-        <v>58</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
updated dating day images + dictionary
</commit_message>
<xml_diff>
--- a/XmlData/Datas/cheeseDictionary.xlsx
+++ b/XmlData/Datas/cheeseDictionary.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Emil\Desktop\projects\GGJ2026\XmlData\Datas\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{634AF970-E859-4399-A306-6AFB9BEE3043}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7D31ED06-B87D-49D5-8BE9-6AE573A6462C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="38280" yWindow="5235" windowWidth="29040" windowHeight="16440" xr2:uid="{53B3FBB6-B116-408D-BCC0-737AAAC6C9D0}"/>
   </bookViews>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="119" uniqueCount="62">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="110" uniqueCount="56">
   <si>
     <t>##var</t>
     <phoneticPr fontId="1" type="noConversion"/>
@@ -186,40 +186,22 @@
     <t>Tax_Evasion</t>
   </si>
   <si>
-    <t>Fraud</t>
-  </si>
-  <si>
     <t>Tax Evasion</t>
   </si>
   <si>
     <t>Visiting</t>
   </si>
   <si>
-    <t>Puerto_Rico</t>
-  </si>
-  <si>
-    <t>Puerto Rico</t>
-  </si>
-  <si>
     <t>Losing</t>
   </si>
   <si>
     <t>Socks</t>
   </si>
   <si>
-    <t>Sesame Street</t>
-  </si>
-  <si>
-    <t>Going_to</t>
-  </si>
-  <si>
-    <t>Sesame_Street</t>
-  </si>
-  <si>
-    <t>Going to</t>
-  </si>
-  <si>
     <t>Salty</t>
+  </si>
+  <si>
+    <t>Jail</t>
   </si>
 </sst>
 </file>
@@ -651,7 +633,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8D4CF470-E9E0-44FF-BA6C-71B5C42FB7B2}">
-  <dimension ref="A1:I34"/>
+  <dimension ref="A1:I31"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="7" bestFit="1" customWidth="1"/>
@@ -983,13 +965,13 @@
         <v>15</v>
       </c>
       <c r="C19" t="s">
-        <v>61</v>
+        <v>54</v>
       </c>
       <c r="D19" t="s">
         <v>37</v>
       </c>
       <c r="E19" t="s">
-        <v>61</v>
+        <v>54</v>
       </c>
     </row>
     <row r="20" spans="2:5">
@@ -1101,7 +1083,7 @@
         <v>10</v>
       </c>
       <c r="E27" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
     </row>
     <row r="28" spans="2:5">
@@ -1109,13 +1091,13 @@
         <v>24</v>
       </c>
       <c r="C28" t="s">
-        <v>50</v>
+        <v>55</v>
       </c>
       <c r="D28" t="s">
         <v>10</v>
       </c>
       <c r="E28" t="s">
-        <v>50</v>
+        <v>55</v>
       </c>
     </row>
     <row r="29" spans="2:5">
@@ -1123,83 +1105,41 @@
         <v>25</v>
       </c>
       <c r="C29" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="D29" t="s">
         <v>47</v>
       </c>
       <c r="E29" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
     </row>
     <row r="30" spans="2:5">
       <c r="B30">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="C30" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="D30" t="s">
-        <v>10</v>
+        <v>47</v>
       </c>
       <c r="E30" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
     </row>
     <row r="31" spans="2:5">
       <c r="B31">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="C31" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="D31" t="s">
-        <v>47</v>
+        <v>10</v>
       </c>
       <c r="E31" t="s">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="32" spans="2:5">
-      <c r="B32">
-        <v>28</v>
-      </c>
-      <c r="C32" t="s">
-        <v>56</v>
-      </c>
-      <c r="D32" t="s">
-        <v>10</v>
-      </c>
-      <c r="E32" t="s">
-        <v>56</v>
-      </c>
-    </row>
-    <row r="33" spans="2:5">
-      <c r="B33">
-        <v>29</v>
-      </c>
-      <c r="C33" t="s">
-        <v>58</v>
-      </c>
-      <c r="D33" t="s">
-        <v>47</v>
-      </c>
-      <c r="E33" t="s">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="34" spans="2:5">
-      <c r="B34">
-        <v>30</v>
-      </c>
-      <c r="C34" t="s">
-        <v>59</v>
-      </c>
-      <c r="D34" t="s">
-        <v>10</v>
-      </c>
-      <c r="E34" t="s">
-        <v>57</v>
+        <v>53</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
separate basic and cheese panel
</commit_message>
<xml_diff>
--- a/XmlData/Datas/cheeseDictionary.xlsx
+++ b/XmlData/Datas/cheeseDictionary.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24334"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Emil\Desktop\projects\GGJ2026\XmlData\Datas\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\yinya\Documents\unityProjects\GGJ2026\XmlData\Datas\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7D31ED06-B87D-49D5-8BE9-6AE573A6462C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B9362846-055C-4185-A98C-EC5E175943C9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="38280" yWindow="5235" windowWidth="29040" windowHeight="16440" xr2:uid="{53B3FBB6-B116-408D-BCC0-737AAAC6C9D0}"/>
+    <workbookView xWindow="-25710" yWindow="-1210" windowWidth="25820" windowHeight="15500" xr2:uid="{53B3FBB6-B116-408D-BCC0-737AAAC6C9D0}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -20,15 +20,12 @@
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
     </ext>
-    <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
-      <xlwcv:version setVersion="1"/>
-    </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="110" uniqueCount="56">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="102" uniqueCount="63">
   <si>
     <t>##var</t>
     <phoneticPr fontId="1" type="noConversion"/>
@@ -168,40 +165,61 @@
     <t>Milk</t>
   </si>
   <si>
+    <t>Cookies</t>
+  </si>
+  <si>
+    <t>Sushi</t>
+  </si>
+  <si>
+    <t>Verb</t>
+  </si>
+  <si>
+    <t>Committing</t>
+  </si>
+  <si>
+    <t>Tax Evasion</t>
+  </si>
+  <si>
+    <t>Losing</t>
+  </si>
+  <si>
+    <t>Socks</t>
+  </si>
+  <si>
+    <t>Salty</t>
+  </si>
+  <si>
+    <t>Jail</t>
+  </si>
+  <si>
+    <t>Visit</t>
+  </si>
+  <si>
+    <t>visiting_jail</t>
+  </si>
+  <si>
+    <t>losing_socks</t>
+  </si>
+  <si>
+    <t>committing_tax_evasion</t>
+  </si>
+  <si>
+    <t>expired_pizza</t>
+  </si>
+  <si>
+    <t>burnt_milk</t>
+  </si>
+  <si>
+    <t>salty_cookies</t>
+  </si>
+  <si>
+    <t>free_sushi</t>
+  </si>
+  <si>
+    <t>frozen_food</t>
+  </si>
+  <si>
     <t>Food</t>
-  </si>
-  <si>
-    <t>Cookies</t>
-  </si>
-  <si>
-    <t>Sushi</t>
-  </si>
-  <si>
-    <t>Verb</t>
-  </si>
-  <si>
-    <t>Committing</t>
-  </si>
-  <si>
-    <t>Tax_Evasion</t>
-  </si>
-  <si>
-    <t>Tax Evasion</t>
-  </si>
-  <si>
-    <t>Visiting</t>
-  </si>
-  <si>
-    <t>Losing</t>
-  </si>
-  <si>
-    <t>Socks</t>
-  </si>
-  <si>
-    <t>Salty</t>
-  </si>
-  <si>
-    <t>Jail</t>
   </si>
 </sst>
 </file>
@@ -337,9 +355,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -377,7 +395,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013 - 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -483,7 +501,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 - 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -625,7 +643,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -633,7 +651,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8D4CF470-E9E0-44FF-BA6C-71B5C42FB7B2}">
-  <dimension ref="A1:I31"/>
+  <dimension ref="A1:I23"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="7" bestFit="1" customWidth="1"/>
@@ -923,7 +941,7 @@
         <v>12</v>
       </c>
       <c r="C16" t="s">
-        <v>38</v>
+        <v>57</v>
       </c>
       <c r="D16" t="s">
         <v>37</v>
@@ -931,13 +949,19 @@
       <c r="E16" t="s">
         <v>38</v>
       </c>
-    </row>
-    <row r="17" spans="2:5">
+      <c r="F16" t="s">
+        <v>10</v>
+      </c>
+      <c r="G16" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="17" spans="2:7">
       <c r="B17">
         <v>13</v>
       </c>
       <c r="C17" t="s">
-        <v>40</v>
+        <v>58</v>
       </c>
       <c r="D17" t="s">
         <v>37</v>
@@ -945,13 +969,19 @@
       <c r="E17" t="s">
         <v>40</v>
       </c>
-    </row>
-    <row r="18" spans="2:5">
+      <c r="F17" t="s">
+        <v>10</v>
+      </c>
+      <c r="G17" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="18" spans="2:7">
       <c r="B18">
         <v>14</v>
       </c>
       <c r="C18" t="s">
-        <v>39</v>
+        <v>61</v>
       </c>
       <c r="D18" t="s">
         <v>37</v>
@@ -959,27 +989,39 @@
       <c r="E18" t="s">
         <v>39</v>
       </c>
-    </row>
-    <row r="19" spans="2:5">
+      <c r="F18" t="s">
+        <v>10</v>
+      </c>
+      <c r="G18" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="19" spans="2:7">
       <c r="B19">
         <v>15</v>
       </c>
       <c r="C19" t="s">
-        <v>54</v>
+        <v>59</v>
       </c>
       <c r="D19" t="s">
         <v>37</v>
       </c>
       <c r="E19" t="s">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="20" spans="2:5">
+        <v>51</v>
+      </c>
+      <c r="F19" t="s">
+        <v>10</v>
+      </c>
+      <c r="G19" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="20" spans="2:7">
       <c r="B20">
         <v>16</v>
       </c>
       <c r="C20" t="s">
-        <v>41</v>
+        <v>60</v>
       </c>
       <c r="D20" t="s">
         <v>37</v>
@@ -987,159 +1029,71 @@
       <c r="E20" t="s">
         <v>41</v>
       </c>
-    </row>
-    <row r="21" spans="2:5">
+      <c r="F20" t="s">
+        <v>10</v>
+      </c>
+      <c r="G20" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="21" spans="2:7">
       <c r="B21">
         <v>17</v>
       </c>
       <c r="C21" t="s">
-        <v>42</v>
+        <v>56</v>
       </c>
       <c r="D21" t="s">
+        <v>46</v>
+      </c>
+      <c r="E21" t="s">
+        <v>47</v>
+      </c>
+      <c r="F21" t="s">
         <v>10</v>
       </c>
-      <c r="E21" t="s">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="22" spans="2:5">
+      <c r="G21" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="22" spans="2:7">
       <c r="B22">
         <v>18</v>
       </c>
       <c r="C22" t="s">
-        <v>43</v>
+        <v>54</v>
       </c>
       <c r="D22" t="s">
+        <v>46</v>
+      </c>
+      <c r="E22" t="s">
+        <v>53</v>
+      </c>
+      <c r="F22" t="s">
         <v>10</v>
       </c>
-      <c r="E22" t="s">
-        <v>43</v>
-      </c>
-    </row>
-    <row r="23" spans="2:5">
+      <c r="G22" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="23" spans="2:7">
       <c r="B23">
         <v>19</v>
       </c>
       <c r="C23" t="s">
-        <v>44</v>
+        <v>55</v>
       </c>
       <c r="D23" t="s">
+        <v>46</v>
+      </c>
+      <c r="E23" t="s">
+        <v>49</v>
+      </c>
+      <c r="F23" t="s">
         <v>10</v>
       </c>
-      <c r="E23" t="s">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="24" spans="2:5">
-      <c r="B24">
-        <v>20</v>
-      </c>
-      <c r="C24" t="s">
-        <v>45</v>
-      </c>
-      <c r="D24" t="s">
-        <v>10</v>
-      </c>
-      <c r="E24" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="25" spans="2:5">
-      <c r="B25">
-        <v>21</v>
-      </c>
-      <c r="C25" t="s">
-        <v>46</v>
-      </c>
-      <c r="D25" t="s">
-        <v>10</v>
-      </c>
-      <c r="E25" t="s">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="26" spans="2:5">
-      <c r="B26">
-        <v>22</v>
-      </c>
-      <c r="C26" t="s">
-        <v>48</v>
-      </c>
-      <c r="D26" t="s">
-        <v>47</v>
-      </c>
-      <c r="E26" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="27" spans="2:5">
-      <c r="B27">
-        <v>23</v>
-      </c>
-      <c r="C27" t="s">
-        <v>49</v>
-      </c>
-      <c r="D27" t="s">
-        <v>10</v>
-      </c>
-      <c r="E27" t="s">
+      <c r="G23" t="s">
         <v>50</v>
-      </c>
-    </row>
-    <row r="28" spans="2:5">
-      <c r="B28">
-        <v>24</v>
-      </c>
-      <c r="C28" t="s">
-        <v>55</v>
-      </c>
-      <c r="D28" t="s">
-        <v>10</v>
-      </c>
-      <c r="E28" t="s">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="29" spans="2:5">
-      <c r="B29">
-        <v>25</v>
-      </c>
-      <c r="C29" t="s">
-        <v>51</v>
-      </c>
-      <c r="D29" t="s">
-        <v>47</v>
-      </c>
-      <c r="E29" t="s">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="30" spans="2:5">
-      <c r="B30">
-        <v>27</v>
-      </c>
-      <c r="C30" t="s">
-        <v>52</v>
-      </c>
-      <c r="D30" t="s">
-        <v>47</v>
-      </c>
-      <c r="E30" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="31" spans="2:5">
-      <c r="B31">
-        <v>28</v>
-      </c>
-      <c r="C31" t="s">
-        <v>53</v>
-      </c>
-      <c r="D31" t="s">
-        <v>10</v>
-      </c>
-      <c r="E31" t="s">
-        <v>53</v>
       </c>
     </row>
   </sheetData>

</xml_diff>